<commit_message>
Updated educators data to include variable data (and changed the conditional formatting)
</commit_message>
<xml_diff>
--- a/data/EDUCATORS 2025.xlsx
+++ b/data/EDUCATORS 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28324"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amsterdamdatacollective-my.sharepoint.com/personal/thomas_b_adc-consulting_com/Documents/Documents/Collective Week/Code/Schooltuinen%20Amsterdam/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AmeliaLindrothADC\Documents\Repositories\Schooltuinen%20Amsterdam\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="910" documentId="11_EA772B53FEDCB482D8F2F109FAFCF9BD061CB40D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74908B06-FFB9-4060-AE77-3165BC9C6BEB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0638FF4-AE60-451F-8982-F561C139A441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="6456" yWindow="4416" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="80">
   <si>
     <t>Medewerker</t>
   </si>
@@ -270,6 +270,12 @@
   </si>
   <si>
     <t>Luanna Jansen</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>Variabel</t>
   </si>
 </sst>
 </file>
@@ -369,7 +375,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="46">
+  <dxfs count="27">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -397,6 +403,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3" tint="0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -432,211 +448,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color theme="3" tint="0.24994659260841701"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -726,26 +542,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{106CB279-B7F9-4066-99A5-AC896AC27FAB}" name="Table1" displayName="Table1" ref="A1:Q44" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{106CB279-B7F9-4066-99A5-AC896AC27FAB}" name="Table1" displayName="Table1" ref="A1:Q44" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A1:Q44" xr:uid="{106CB279-B7F9-4066-99A5-AC896AC27FAB}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{AA185061-3FA7-4C2E-9AB8-B17CAF7C8F92}" name="Tuinlocatie" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{4553C0AA-C4EE-4E03-85B9-B3FDFCAF69D5}" name="Medewerker" dataDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{69D44180-F9D6-4C20-944F-75CCDEB26201}" name="maandag, 09.00 - 10.30" dataDxfId="41"/>
-    <tableColumn id="4" xr3:uid="{A8C0A567-ED10-4E56-9A64-2E7E614B4307}" name="maandag, 10.45 - 12.15" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{9390CB88-79B6-4667-ACF3-EFFEE0918B14}" name="maandag, 13.30 - 15.00" dataDxfId="39"/>
-    <tableColumn id="6" xr3:uid="{053A913E-5869-4B77-97E2-9EF8214C6A4A}" name="dinsdag, 09.00 - 10.30" dataDxfId="38"/>
-    <tableColumn id="7" xr3:uid="{CC1BAAF6-4711-429F-9D52-3FBEC2058514}" name="dinsdag, 10.45 - 12.15" dataDxfId="37"/>
-    <tableColumn id="8" xr3:uid="{CB04C8EA-5D9D-4E5D-B3D7-63B5275DFADF}" name="dinsdag, 13.30 - 15.00" dataDxfId="36"/>
-    <tableColumn id="9" xr3:uid="{56459540-AB9E-47AC-BABB-6975F906061F}" name="woensdag, 09.00 - 10.30" dataDxfId="35"/>
-    <tableColumn id="10" xr3:uid="{CFDF740E-8FFD-4871-9B27-E67363F78C65}" name="woensdag, 10.45 - 12.15" dataDxfId="34"/>
-    <tableColumn id="11" xr3:uid="{5E9E0784-AB14-4972-9617-C3940DF01C6D}" name="woensdag, 13.30 - 15.00" dataDxfId="33"/>
-    <tableColumn id="12" xr3:uid="{010732F2-830D-4971-9D1E-F7199948C5F1}" name="donderdag, 09.00 - 10.30" dataDxfId="32"/>
-    <tableColumn id="13" xr3:uid="{460B6053-F08D-47D7-9282-8EB02C0C4511}" name="donderdag, 10.45 - 12.15" dataDxfId="31"/>
-    <tableColumn id="14" xr3:uid="{F9888B0F-530F-403B-AEC4-9EEEA0549C54}" name="donderdag, 13.30 - 15.00" dataDxfId="30"/>
-    <tableColumn id="15" xr3:uid="{8EC093AC-4D5C-4CBC-8948-48791EE7F218}" name="vrijdag, 09.00 - 10.30" dataDxfId="29"/>
-    <tableColumn id="16" xr3:uid="{FC6FA66D-ED39-4C2B-A148-113F55D95268}" name="vrijdag, 10.45 - 12.15" dataDxfId="28"/>
-    <tableColumn id="17" xr3:uid="{4FE55670-2894-43DA-A666-433FAB1F5423}" name="vrijdag, 13.30 - 15.00" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{AA185061-3FA7-4C2E-9AB8-B17CAF7C8F92}" name="Tuinlocatie" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{4553C0AA-C4EE-4E03-85B9-B3FDFCAF69D5}" name="Medewerker" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{69D44180-F9D6-4C20-944F-75CCDEB26201}" name="maandag, 09.00 - 10.30" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{A8C0A567-ED10-4E56-9A64-2E7E614B4307}" name="maandag, 10.45 - 12.15" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{9390CB88-79B6-4667-ACF3-EFFEE0918B14}" name="maandag, 13.30 - 15.00" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{053A913E-5869-4B77-97E2-9EF8214C6A4A}" name="dinsdag, 09.00 - 10.30" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{CC1BAAF6-4711-429F-9D52-3FBEC2058514}" name="dinsdag, 10.45 - 12.15" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{CB04C8EA-5D9D-4E5D-B3D7-63B5275DFADF}" name="dinsdag, 13.30 - 15.00" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{56459540-AB9E-47AC-BABB-6975F906061F}" name="woensdag, 09.00 - 10.30" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{CFDF740E-8FFD-4871-9B27-E67363F78C65}" name="woensdag, 10.45 - 12.15" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{5E9E0784-AB14-4972-9617-C3940DF01C6D}" name="woensdag, 13.30 - 15.00" dataDxfId="14"/>
+    <tableColumn id="12" xr3:uid="{010732F2-830D-4971-9D1E-F7199948C5F1}" name="donderdag, 09.00 - 10.30" dataDxfId="13"/>
+    <tableColumn id="13" xr3:uid="{460B6053-F08D-47D7-9282-8EB02C0C4511}" name="donderdag, 10.45 - 12.15" dataDxfId="12"/>
+    <tableColumn id="14" xr3:uid="{F9888B0F-530F-403B-AEC4-9EEEA0549C54}" name="donderdag, 13.30 - 15.00" dataDxfId="11"/>
+    <tableColumn id="15" xr3:uid="{8EC093AC-4D5C-4CBC-8948-48791EE7F218}" name="vrijdag, 09.00 - 10.30" dataDxfId="10"/>
+    <tableColumn id="16" xr3:uid="{FC6FA66D-ED39-4C2B-A148-113F55D95268}" name="vrijdag, 10.45 - 12.15" dataDxfId="9"/>
+    <tableColumn id="17" xr3:uid="{4FE55670-2894-43DA-A666-433FAB1F5423}" name="vrijdag, 13.30 - 15.00" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1080,20 +896,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="25" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="23.90625" bestFit="1" customWidth="1"/>
     <col min="9" max="11" width="26" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="22.6328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>53</v>
       </c>
@@ -1154,7 +970,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>54</v>
       </c>
@@ -1206,14 +1022,14 @@
       <c r="Q2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="T2" t="s">
+      <c r="T2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="U2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>54</v>
       </c>
@@ -1265,14 +1081,14 @@
       <c r="Q3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="T3" t="s">
+      <c r="T3" s="2" t="s">
         <v>51</v>
       </c>
       <c r="U3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>55</v>
       </c>
@@ -1324,14 +1140,14 @@
       <c r="Q4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="T4" t="s">
+      <c r="T4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="U4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>55</v>
       </c>
@@ -1383,8 +1199,14 @@
       <c r="Q5" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="T5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="U5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>55</v>
       </c>
@@ -1437,7 +1259,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>56</v>
       </c>
@@ -1490,7 +1312,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>56</v>
       </c>
@@ -1543,7 +1365,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>57</v>
       </c>
@@ -1596,7 +1418,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>57</v>
       </c>
@@ -1649,7 +1471,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>57</v>
       </c>
@@ -1702,7 +1524,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>57</v>
       </c>
@@ -1755,7 +1577,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>59</v>
       </c>
@@ -1808,7 +1630,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>59</v>
       </c>
@@ -1861,7 +1683,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>59</v>
       </c>
@@ -1914,7 +1736,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>59</v>
       </c>
@@ -1967,7 +1789,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>60</v>
       </c>
@@ -2020,7 +1842,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>60</v>
       </c>
@@ -2073,7 +1895,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>60</v>
       </c>
@@ -2126,7 +1948,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>61</v>
       </c>
@@ -2179,7 +2001,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>61</v>
       </c>
@@ -2232,7 +2054,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>61</v>
       </c>
@@ -2285,7 +2107,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>61</v>
       </c>
@@ -2338,7 +2160,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>62</v>
       </c>
@@ -2391,7 +2213,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>62</v>
       </c>
@@ -2444,7 +2266,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>63</v>
       </c>
@@ -2497,7 +2319,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>63</v>
       </c>
@@ -2550,7 +2372,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>63</v>
       </c>
@@ -2603,7 +2425,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>64</v>
       </c>
@@ -2656,7 +2478,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>64</v>
       </c>
@@ -2709,7 +2531,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>64</v>
       </c>
@@ -2762,7 +2584,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>64</v>
       </c>
@@ -2815,7 +2637,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>64</v>
       </c>
@@ -2868,7 +2690,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>64</v>
       </c>
@@ -2921,7 +2743,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>65</v>
       </c>
@@ -2974,7 +2796,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>65</v>
       </c>
@@ -3027,7 +2849,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>65</v>
       </c>
@@ -3080,7 +2902,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>65</v>
       </c>
@@ -3133,7 +2955,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>66</v>
       </c>
@@ -3186,7 +3008,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>66</v>
       </c>
@@ -3239,7 +3061,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>66</v>
       </c>
@@ -3292,7 +3114,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>68</v>
       </c>
@@ -3345,7 +3167,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>68</v>
       </c>
@@ -3398,7 +3220,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>68</v>
       </c>
@@ -3452,107 +3274,32 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:E5">
-    <cfRule type="expression" dxfId="26" priority="22">
-      <formula>C5="M"</formula>
+  <conditionalFormatting sqref="C2:Q1048576">
+    <cfRule type="cellIs" dxfId="7" priority="17" operator="equal">
+      <formula>"V"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="23">
-      <formula>C5="U"</formula>
+    <cfRule type="cellIs" dxfId="6" priority="18" operator="equal">
+      <formula>"O"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="24">
-      <formula>C5="X"</formula>
+    <cfRule type="cellIs" dxfId="5" priority="19" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="20" operator="equal">
+      <formula>"B"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:H4">
-    <cfRule type="expression" dxfId="23" priority="37">
-      <formula>C4="M"</formula>
+  <conditionalFormatting sqref="T2:T5">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+      <formula>"V"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="38">
-      <formula>C4="U"</formula>
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+      <formula>"O"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="39">
-      <formula>C4="X"</formula>
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+      <formula>"N"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C9:Q9">
-    <cfRule type="expression" dxfId="20" priority="1">
-      <formula>C9="M"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="19" priority="2">
-      <formula>C9="U"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="18" priority="3">
-      <formula>C9="X"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:U15 C16:S16 U16 C17:U104">
-    <cfRule type="expression" dxfId="17" priority="42">
-      <formula>C2="B"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:U15 C16:S16 U16 C17:U118">
-    <cfRule type="expression" dxfId="16" priority="41">
-      <formula>C2="N"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:U15 C16:S16 U16 C17:U123">
-    <cfRule type="expression" dxfId="15" priority="40">
-      <formula>C2="O"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F5:H5">
-    <cfRule type="expression" dxfId="14" priority="19">
-      <formula>F5="M"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="20">
-      <formula>F5="U"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="21">
-      <formula>F5="X"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I4:J5">
-    <cfRule type="expression" dxfId="11" priority="16">
-      <formula>I4="M"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="17">
-      <formula>I4="U"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="18">
-      <formula>I4="X"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K4:K5">
-    <cfRule type="expression" dxfId="8" priority="10">
-      <formula>K4="M"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="11">
-      <formula>K4="U"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="12">
-      <formula>K4="X"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L4:N5">
-    <cfRule type="expression" dxfId="5" priority="7">
-      <formula>L4="M"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="8">
-      <formula>L4="U"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="9">
-      <formula>L4="X"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O4:Q5">
-    <cfRule type="expression" dxfId="2" priority="4">
-      <formula>O4="M"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="5">
-      <formula>O4="U"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="6">
-      <formula>O4="X"</formula>
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+      <formula>"B"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Refactor garden scheduling constraints and update configuration settings
</commit_message>
<xml_diff>
--- a/data/EDUCATORS 2025.xlsx
+++ b/data/EDUCATORS 2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakob/Documents/ADC/projects/Schooltuinen%20Amsterdam/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DAB3DA7-3040-4348-9FB2-FFE7BAAA703D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{211D7BB7-A9EF-564C-B33A-ED9074F567C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,51 +42,6 @@
     <t>Medewerker</t>
   </si>
   <si>
-    <t>maandag, 09.00 - 10.30</t>
-  </si>
-  <si>
-    <t>maandag, 10.45 - 12.15</t>
-  </si>
-  <si>
-    <t>maandag, 13.30 - 15.00</t>
-  </si>
-  <si>
-    <t>dinsdag, 09.00 - 10.30</t>
-  </si>
-  <si>
-    <t>dinsdag, 10.45 - 12.15</t>
-  </si>
-  <si>
-    <t>dinsdag, 13.30 - 15.00</t>
-  </si>
-  <si>
-    <t>woensdag, 09.00 - 10.30</t>
-  </si>
-  <si>
-    <t>woensdag, 10.45 - 12.15</t>
-  </si>
-  <si>
-    <t>woensdag, 13.30 - 15.00</t>
-  </si>
-  <si>
-    <t>donderdag, 09.00 - 10.30</t>
-  </si>
-  <si>
-    <t>donderdag, 10.45 - 12.15</t>
-  </si>
-  <si>
-    <t>donderdag, 13.30 - 15.00</t>
-  </si>
-  <si>
-    <t>vrijdag, 09.00 - 10.30</t>
-  </si>
-  <si>
-    <t>vrijdag, 10.45 - 12.15</t>
-  </si>
-  <si>
-    <t>vrijdag, 13.30 - 15.00</t>
-  </si>
-  <si>
     <t>Code</t>
   </si>
   <si>
@@ -277,6 +232,51 @@
   </si>
   <si>
     <t>Variabel</t>
+  </si>
+  <si>
+    <t>maandag, 09:00-10:30</t>
+  </si>
+  <si>
+    <t>maandag, 10:45-12:15</t>
+  </si>
+  <si>
+    <t>maandag, 13:30-15:00</t>
+  </si>
+  <si>
+    <t>dinsdag, 09:00-10:30</t>
+  </si>
+  <si>
+    <t>dinsdag, 10:45-12:15</t>
+  </si>
+  <si>
+    <t>dinsdag, 13:30-15:00</t>
+  </si>
+  <si>
+    <t>woensdag, 09:00-10:30</t>
+  </si>
+  <si>
+    <t>woensdag, 10:45-12:15</t>
+  </si>
+  <si>
+    <t>woensdag, 13:30-15:00</t>
+  </si>
+  <si>
+    <t>donderdag, 09:00-10:30</t>
+  </si>
+  <si>
+    <t>donderdag, 10:45-12:15</t>
+  </si>
+  <si>
+    <t>donderdag, 13:30-15:00</t>
+  </si>
+  <si>
+    <t>vrijdag, 09:00-10:30</t>
+  </si>
+  <si>
+    <t>vrijdag, 10:45-12:15</t>
+  </si>
+  <si>
+    <t>vrijdag, 13:30-15:00</t>
   </si>
 </sst>
 </file>
@@ -372,7 +372,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -551,21 +551,21 @@
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{AA185061-3FA7-4C2E-9AB8-B17CAF7C8F92}" name="Tuinlocatie" dataDxfId="24"/>
     <tableColumn id="2" xr3:uid="{4553C0AA-C4EE-4E03-85B9-B3FDFCAF69D5}" name="Medewerker" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{69D44180-F9D6-4C20-944F-75CCDEB26201}" name="maandag, 09.00 - 10.30" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{A8C0A567-ED10-4E56-9A64-2E7E614B4307}" name="maandag, 10.45 - 12.15" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{9390CB88-79B6-4667-ACF3-EFFEE0918B14}" name="maandag, 13.30 - 15.00" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{053A913E-5869-4B77-97E2-9EF8214C6A4A}" name="dinsdag, 09.00 - 10.30" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{CC1BAAF6-4711-429F-9D52-3FBEC2058514}" name="dinsdag, 10.45 - 12.15" dataDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{CB04C8EA-5D9D-4E5D-B3D7-63B5275DFADF}" name="dinsdag, 13.30 - 15.00" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{56459540-AB9E-47AC-BABB-6975F906061F}" name="woensdag, 09.00 - 10.30" dataDxfId="16"/>
-    <tableColumn id="10" xr3:uid="{CFDF740E-8FFD-4871-9B27-E67363F78C65}" name="woensdag, 10.45 - 12.15" dataDxfId="15"/>
-    <tableColumn id="11" xr3:uid="{5E9E0784-AB14-4972-9617-C3940DF01C6D}" name="woensdag, 13.30 - 15.00" dataDxfId="14"/>
-    <tableColumn id="12" xr3:uid="{010732F2-830D-4971-9D1E-F7199948C5F1}" name="donderdag, 09.00 - 10.30" dataDxfId="13"/>
-    <tableColumn id="13" xr3:uid="{460B6053-F08D-47D7-9282-8EB02C0C4511}" name="donderdag, 10.45 - 12.15" dataDxfId="12"/>
-    <tableColumn id="14" xr3:uid="{F9888B0F-530F-403B-AEC4-9EEEA0549C54}" name="donderdag, 13.30 - 15.00" dataDxfId="11"/>
-    <tableColumn id="15" xr3:uid="{8EC093AC-4D5C-4CBC-8948-48791EE7F218}" name="vrijdag, 09.00 - 10.30" dataDxfId="10"/>
-    <tableColumn id="16" xr3:uid="{FC6FA66D-ED39-4C2B-A148-113F55D95268}" name="vrijdag, 10.45 - 12.15" dataDxfId="9"/>
-    <tableColumn id="17" xr3:uid="{4FE55670-2894-43DA-A666-433FAB1F5423}" name="vrijdag, 13.30 - 15.00" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{69D44180-F9D6-4C20-944F-75CCDEB26201}" name="maandag, 09:00-10:30" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{A8C0A567-ED10-4E56-9A64-2E7E614B4307}" name="maandag, 10:45-12:15" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{9390CB88-79B6-4667-ACF3-EFFEE0918B14}" name="maandag, 13:30-15:00" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{053A913E-5869-4B77-97E2-9EF8214C6A4A}" name="dinsdag, 09:00-10:30" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{CC1BAAF6-4711-429F-9D52-3FBEC2058514}" name="dinsdag, 10:45-12:15" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{CB04C8EA-5D9D-4E5D-B3D7-63B5275DFADF}" name="dinsdag, 13:30-15:00" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{56459540-AB9E-47AC-BABB-6975F906061F}" name="woensdag, 09:00-10:30" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{CFDF740E-8FFD-4871-9B27-E67363F78C65}" name="woensdag, 10:45-12:15" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{5E9E0784-AB14-4972-9617-C3940DF01C6D}" name="woensdag, 13:30-15:00" dataDxfId="14"/>
+    <tableColumn id="12" xr3:uid="{010732F2-830D-4971-9D1E-F7199948C5F1}" name="donderdag, 09:00-10:30" dataDxfId="13"/>
+    <tableColumn id="13" xr3:uid="{460B6053-F08D-47D7-9282-8EB02C0C4511}" name="donderdag, 10:45-12:15" dataDxfId="12"/>
+    <tableColumn id="14" xr3:uid="{F9888B0F-530F-403B-AEC4-9EEEA0549C54}" name="donderdag, 13:30-15:00" dataDxfId="11"/>
+    <tableColumn id="15" xr3:uid="{8EC093AC-4D5C-4CBC-8948-48791EE7F218}" name="vrijdag, 09:00-10:30" dataDxfId="10"/>
+    <tableColumn id="16" xr3:uid="{FC6FA66D-ED39-4C2B-A148-113F55D95268}" name="vrijdag, 10:45-12:15" dataDxfId="9"/>
+    <tableColumn id="17" xr3:uid="{4FE55670-2894-43DA-A666-433FAB1F5423}" name="vrijdag, 13:30-15:00" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -902,2334 +902,2334 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2</v>
+        <v>66</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>3</v>
+        <v>67</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>5</v>
+        <v>69</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>6</v>
+        <v>70</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>7</v>
+        <v>71</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>9</v>
+        <v>73</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>10</v>
+        <v>74</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>11</v>
+        <v>75</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>12</v>
+        <v>76</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>13</v>
+        <v>77</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>14</v>
+        <v>78</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>15</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q23" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q24" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q25" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q27" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q28" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q29" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O30" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q30" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q31" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q32" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P34" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q34" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P35" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q35" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q36" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q37" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q38" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q39" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q40" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="L41" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q41" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O43" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="O44" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -3261,42 +3261,42 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -3319,6 +3319,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A42C61A6A2258C40BDFECD0BFE7AB149" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2f2bd0a4d5f789eebc9e9c32900f24e4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5f414dda-f070-4b2c-a6a7-701907f758f3" xmlns:ns3="9701c0c3-e6e0-4347-a789-f10f63287cd9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a00c581b083e96fa0d5c8560d2b4ce04" ns2:_="" ns3:_="">
     <xsd:import namespace="5f414dda-f070-4b2c-a6a7-701907f758f3"/>
@@ -3573,15 +3582,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3594,6 +3594,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6D8E0F6-4DD4-4592-A255-F16C2E6BC8B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0E4613B-97A9-4B3A-B03C-2E3DF7560EC6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3612,14 +3620,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6D8E0F6-4DD4-4592-A255-F16C2E6BC8B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A4D735E-97E2-4C58-B210-67FF382FAF05}">
   <ds:schemaRefs>

</xml_diff>